<commit_message>
Update LinkedEye_Complete_Flow status to reflect deployments
Module Flow Master: 16 of 28 modules now "Deployed"
K8s Deployment: updated with actual EKS namespaces and pod counts
Tech Stack: deployment column updated with actual locations (EKS/on-prem)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LinkedEye_Complete_Flow.xlsx
+++ b/LinkedEye_Complete_Flow.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,11 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +94,12 @@
         <fgColor rgb="00CCE5FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -142,6 +151,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -645,9 +657,9 @@
           <t>Anomaly detection on metrics using statistical models</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -713,9 +725,9 @@
           <t>Predictive scaling recommendations</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -847,9 +859,9 @@
           <t>Log pattern analysis, error clustering</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -915,9 +927,9 @@
           <t>Alert correlation, noise reduction, dedup ML</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -986,9 +998,9 @@
           <t>AI Auto-classify (Mistral-7B), AI Auto-assign, Similar incident search (BGE embeddings + cosine), NL incident creation, RCA suggestion (Qwen3-32B)</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1053,9 +1065,9 @@
           <t>Predictive SLA breach probability</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1536,9 +1548,9 @@
           <t>Mistral-7B: classification, Qwen3-32B: RCA generation, BGE: embeddings, ChromaDB: vector store</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1603,9 +1615,9 @@
           <t>Llama3.1:70b (conversation), Mistral-7B (classification), BGE (RAG retrieval)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1738,9 +1750,9 @@
           <t>ML classification model, workload-aware assignment algorithm</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1876,9 +1888,9 @@
           <t>Whisper STT (94.2% accuracy), Qwen3 LLM (91.8%), Tamil voice (88.5%)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2218,9 +2230,9 @@
           <t>Anomalous login detection</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2287,9 +2299,9 @@
           <t>AI-generated daily summary, trend analysis</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2354,9 +2366,9 @@
           <t>AI enrichment worker pipeline</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2490,9 +2502,9 @@
           <t>Auto-provisioning recommendations</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>Deployed</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -6857,7 +6869,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-frontend namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -6887,7 +6899,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Bundled with Next.js</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -6917,7 +6929,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Build-time compilation</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6959,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Client-side rendering</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -6977,7 +6989,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Auto-reconnect, fallback polling</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7019,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-api namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7049,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Cluster mode (PM2)</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7067,7 +7079,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Horizontal scaling via Redis pub/sub</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7097,7 +7109,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Redis-backed, multiple workers</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7139,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Migrations, model validations</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7157,7 +7169,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-db namespace, streaming replication</t>
+          <t>Deployed: EKS (le-postgres) + on-prem</t>
         </is>
       </c>
     </row>
@@ -7187,7 +7199,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-cache namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7229,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-ai namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7259,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-ai namespace, GPU node</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7289,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-ai namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7319,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-ai namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7349,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-ai namespace</t>
+          <t>Deployed: on-prem (fs-linkedeye)</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7379,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>K8s: monitoring namespace</t>
+          <t>Deployed: EKS (le-monitoring)</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7409,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>K8s: monitoring namespace</t>
+          <t>Deployed: EKS (le-monitoring)</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7439,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>K8s: monitoring namespace</t>
+          <t>Deployed: EKS (le-monitoring)</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7469,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-auth namespace</t>
+          <t>Deployed: EKS (le-keycloak)</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7499,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-automation namespace</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -7517,7 +7529,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Control node in K8s</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7559,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Cloud API</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
@@ -7577,7 +7589,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-comms namespace</t>
+          <t>Deployed: EKS (le-monitoring)</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7619,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>AWS EKS + self-hosted nodes</t>
+          <t>Deployed: EKS + on-prem (hybrid nodes)</t>
         </is>
       </c>
     </row>
@@ -7637,7 +7649,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>All services containerized</t>
+          <t>Deployed: EKS + on-prem</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7679,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>GitOps workflow</t>
+          <t>Not used (bash scripts instead)</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7709,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>K8s: linkedeye-storage namespace</t>
+          <t>Deployed: EKS (le-minio)</t>
         </is>
       </c>
     </row>
@@ -8851,17 +8863,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Next.js dashboard, Nginx ingress</t>
+          <t>React + Nginx (le-frontend)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>500m/512Mi per pod</t>
+          <t>100m/64Mi</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -8871,7 +8883,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CDN for static assets</t>
+          <t>Deployed on on-prem cluster (fs-linkedeye ns)</t>
         </is>
       </c>
     </row>
@@ -8886,27 +8898,27 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Express.js API, Socket.IO server, BullMQ workers (ai-enrichment, sla-check, email-digest, report-gen)</t>
+          <t>Node.js Express API + Socket.IO</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>3-5 (HPA)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>1000m/1Gi per pod</t>
+          <t>250m/256Mi</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Temp storage for file uploads</t>
+          <t>Temp uploads</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Auto-scale on CPU &gt; 70%</t>
+          <t>Deployed on on-prem cluster (fs-linkedeye ns)</t>
         </is>
       </c>
     </row>
@@ -8916,32 +8928,32 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>linkedeye-db</t>
+          <t>le-postgres</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL (primary + read replica), Redis Sentinel (3 nodes)</t>
+          <t>PostgreSQL 16</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2 (PG) + 3 (Redis)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2000m/4Gi (PG), 500m/1Gi (Redis)</t>
+          <t>500m/1Gi</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>100Gi PVC (PG), 10Gi (Redis AOF)</t>
+          <t>EBS PVC 50Gi</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Streaming replication, Sentinel HA</t>
+          <t>Deployed on EKS (le-postgres ns)</t>
         </is>
       </c>
     </row>
@@ -8951,32 +8963,32 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-ai</t>
+          <t>le-monitoring</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Ollama (3 models), Flowise (6 chatflows), ChromaDB, HuggingFace TEI, Whisper</t>
+          <t>Prometheus, Grafana :30090, Alertmanager</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1-2 per service</t>
+          <t>7 pods</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>4000m/8Gi (Ollama GPU), 1000m/2Gi (others)</t>
+          <t>2Gi (Prometheus)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>50Gi (model storage), 20Gi (ChromaDB)</t>
+          <t>50Gi PVC</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>GPU node required for Ollama</t>
+          <t>Deployed on EKS (le-monitoring ns)</t>
         </is>
       </c>
     </row>
@@ -8986,32 +8998,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>linkedeye-auth</t>
+          <t>le-keycloak</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Keycloak (HA), realm: linkedeye-prod</t>
+          <t>Keycloak SSO</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1000m/2Gi per pod</t>
+          <t>500m/512Mi</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL backend (shared)</t>
+          <t>PostgreSQL backend</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>OIDC + PKCE, MFA TOTP</t>
+          <t>Deployed on EKS (le-keycloak ns)</t>
         </is>
       </c>
     </row>
@@ -9021,32 +9033,32 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-automation</t>
+          <t>le-jenkins</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>n8n (14 workflows), Ansible control node</t>
+          <t>Jenkins CI/CD</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>500m/1Gi per service</t>
+          <t>500m/1Gi</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>5Gi (workflow data)</t>
+          <t>EBS PVC</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Event-driven scaling</t>
+          <t>Deployed on EKS (le-jenkins ns)</t>
         </is>
       </c>
     </row>
@@ -9056,32 +9068,32 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>linkedeye-comms</t>
+          <t>le-minio</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Chatwoot (omni-channel), Email service</t>
+          <t>MinIO S3 Storage</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>500m/1Gi per pod</t>
+          <t>256m/512Mi</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>10Gi (message history)</t>
+          <t>EBS PVC</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>WhatsApp/Web/Email gateway</t>
+          <t>Deployed on EKS (le-minio ns)</t>
         </is>
       </c>
     </row>
@@ -9091,32 +9103,32 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>linkedeye-storage</t>
+          <t>le-argocd</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>MinIO (S3-compatible object storage)</t>
+          <t>ArgoCD GitOps</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3 (distributed)</t>
+          <t>4 pods</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>500m/1Gi per pod</t>
+          <t>256m/256Mi</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>200Gi (attachments, recordings, snapshots)</t>
+          <t>No PVC</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Erasure coding for durability</t>
+          <t>Deployed on EKS (le-argocd ns)</t>
         </is>
       </c>
     </row>
@@ -9126,32 +9138,32 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>monitoring</t>
+          <t>le-harbor</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Prometheus, Alertmanager, Loki, Promtail, Grafana</t>
+          <t>Harbor Container Registry</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1-2 per service</t>
+          <t>5 pods</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2000m/4Gi (Prometheus), 1000m/2Gi (others)</t>
+          <t>256m/512Mi</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>100Gi (Prometheus TSDB), 50Gi (Loki)</t>
+          <t>EBS PVC</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Shared across tenants, org isolation in Grafana</t>
+          <t>Deployed on EKS (le-harbor ns)</t>
         </is>
       </c>
     </row>

</xml_diff>